<commit_message>
update file, cuze xcel was out dated
</commit_message>
<xml_diff>
--- a/TextPad7/TextPad_Test_Report_and_Bug_report_template.xlsx
+++ b/TextPad7/TextPad_Test_Report_and_Bug_report_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\opilane\source\repos\Christoferkrabbi\TextPad7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0191F610-F46A-43C6-898E-F0EDB6AB2380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4A1B537-D11F-4F1A-A282-3D58DC1A3785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14445" yWindow="1815" windowWidth="22215" windowHeight="16455" firstSheet="5" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14790" yWindow="2220" windowWidth="22215" windowHeight="16455" firstSheet="9" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Report" sheetId="11" r:id="rId1"/>
@@ -29,6 +29,9 @@
     <sheet name="Bug 13" sheetId="16" r:id="rId14"/>
     <sheet name="Bug 14" sheetId="17" r:id="rId15"/>
     <sheet name="Bug 15" sheetId="18" r:id="rId16"/>
+    <sheet name="Bug 16" sheetId="19" r:id="rId17"/>
+    <sheet name="Bug 17" sheetId="20" r:id="rId18"/>
+    <sheet name="Bug 18" sheetId="21" r:id="rId19"/>
   </sheets>
   <calcPr calcId="125725"/>
   <extLst>
@@ -40,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="63">
   <si>
     <t>Product:</t>
   </si>
@@ -279,6 +282,33 @@
   </si>
   <si>
     <t>Misplaced selection box in 'Print' window</t>
+  </si>
+  <si>
+    <t>misaligned 'Zoom in' in 'Print preview'</t>
+  </si>
+  <si>
+    <t>Steps to reproduce: 
+1. Launch 'TextPad'
+2. Open any file with text in it
+3. go to 'File' and select 'Print preview'
+Expected result:
+There are no misalignments
+Actual result:
+There are misalignments</t>
+  </si>
+  <si>
+    <t>The option 'Print' gives an error when using a file with only one page worth of text</t>
+  </si>
+  <si>
+    <t>Steps to reproduce: 
+1. Launch 'TextPad'
+2. Open any file with text in it
+3. go to 'File' and select 'Print preview'
+4. Press 'print' 
+Expected result:
+Pressing the button brings up the 'Print' window
+Actual result:
+The program closed and gave an error</t>
   </si>
 </sst>
 </file>
@@ -1447,6 +1477,121 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>285750</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>6125398</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>2467279</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Pilt 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CEEA6B83-3A31-4295-BF59-69A2031DDBC7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1638300" y="4124325"/>
+          <a:ext cx="5896798" cy="2181529"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2933700</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>409575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>3800475</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>809625</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="Ristkülik 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AAC1B612-E9AA-4F68-ADBB-06F1AF292E62}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4343400" y="4248150"/>
+          <a:ext cx="866775" cy="400050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="et-EE" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
@@ -3571,7 +3716,9 @@
         <v>21</v>
       </c>
       <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
+      <c r="D3" s="21">
+        <v>7</v>
+      </c>
     </row>
     <row r="4" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
@@ -4080,7 +4227,9 @@
       <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="30"/>
+      <c r="C2" s="30">
+        <v>13</v>
+      </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
@@ -4118,13 +4267,17 @@
       <c r="B7" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="28"/>
+      <c r="C7" s="28" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="8" spans="2:3" ht="196.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="29"/>
+      <c r="C8" s="29" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="9" spans="2:3" ht="211.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="6" t="s">
@@ -4134,6 +4287,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -4151,7 +4306,9 @@
       <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="30"/>
+      <c r="C2" s="30">
+        <v>14</v>
+      </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
@@ -4189,13 +4346,17 @@
       <c r="B7" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="28"/>
+      <c r="C7" s="28" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="8" spans="2:3" ht="196.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="29"/>
+      <c r="C8" s="29" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="9" spans="2:3" ht="211.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="6" t="s">
@@ -4222,7 +4383,228 @@
       <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="30"/>
+      <c r="C2" s="30">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="28"/>
+    </row>
+    <row r="8" spans="2:3" ht="196.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="29"/>
+    </row>
+    <row r="9" spans="2:3" ht="211.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EE21A4C-DCB3-4F52-AA79-A54B46CC1859}">
+  <dimension ref="B1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="109.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="30">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="28"/>
+    </row>
+    <row r="8" spans="2:3" ht="196.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="29"/>
+    </row>
+    <row r="9" spans="2:3" ht="211.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81C2CB9D-D56B-45C1-AA57-FDF81708DD81}">
+  <dimension ref="B1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="109.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="30">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="28"/>
+    </row>
+    <row r="8" spans="2:3" ht="196.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="29"/>
+    </row>
+    <row r="9" spans="2:3" ht="211.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B5790E9-2382-4FDE-8518-91E6948A00AA}">
+  <dimension ref="B1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="109.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="30">
+        <v>18</v>
+      </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">

</xml_diff>